<commit_message>
Added set logos, updated metadata file with set logo filenames, added chart_style for branding and made first meta share visual
</commit_message>
<xml_diff>
--- a/metadata/metadata.xlsx
+++ b/metadata/metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madis\Documents\pokemon_scraper\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86E36E6-4B6F-455B-B29A-A1B31248EE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0DB85E6-0613-4051-92D8-8FF68D36BB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-2460" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tournaments" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="233">
   <si>
     <t>tournament_id</t>
   </si>
@@ -660,6 +660,75 @@
   </si>
   <si>
     <t>Hydreigon ex</t>
+  </si>
+  <si>
+    <t>asset_filename</t>
+  </si>
+  <si>
+    <t>svi.png</t>
+  </si>
+  <si>
+    <t>pal.png</t>
+  </si>
+  <si>
+    <t>obf.png</t>
+  </si>
+  <si>
+    <t>mew.png</t>
+  </si>
+  <si>
+    <t>par.png</t>
+  </si>
+  <si>
+    <t>paf.png</t>
+  </si>
+  <si>
+    <t>tef.png</t>
+  </si>
+  <si>
+    <t>twm.png</t>
+  </si>
+  <si>
+    <t>sfa.png</t>
+  </si>
+  <si>
+    <t>scr.png</t>
+  </si>
+  <si>
+    <t>ssp.png</t>
+  </si>
+  <si>
+    <t>pre.png</t>
+  </si>
+  <si>
+    <t>jtg.png</t>
+  </si>
+  <si>
+    <t>dri.png</t>
+  </si>
+  <si>
+    <t>blk.png</t>
+  </si>
+  <si>
+    <t>wht.png</t>
+  </si>
+  <si>
+    <t>meg.png</t>
+  </si>
+  <si>
+    <t>pfl.png</t>
+  </si>
+  <si>
+    <t>asc.png</t>
+  </si>
+  <si>
+    <t>por.png</t>
+  </si>
+  <si>
+    <t>cri.png</t>
+  </si>
+  <si>
+    <t>pbl.png</t>
   </si>
 </sst>
 </file>
@@ -1125,21 +1194,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0D6416A-2744-408B-ACBE-6C19FD322B6D}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>78</v>
       </c>
@@ -1153,10 +1224,13 @@
         <v>24</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1169,11 +1243,11 @@
       <c r="D2" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>45015</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1186,11 +1260,11 @@
       <c r="D3" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="2">
         <v>45015</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1203,11 +1277,14 @@
       <c r="D4" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" t="s">
+        <v>211</v>
+      </c>
+      <c r="F4" s="2">
         <v>45016</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1220,11 +1297,14 @@
       <c r="D5" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" t="s">
+        <v>212</v>
+      </c>
+      <c r="F5" s="2">
         <v>45086</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1237,11 +1317,14 @@
       <c r="D6" t="s">
         <v>64</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" t="s">
+        <v>213</v>
+      </c>
+      <c r="F6" s="2">
         <v>45149</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1254,11 +1337,14 @@
       <c r="D7" t="s">
         <v>65</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" t="s">
+        <v>214</v>
+      </c>
+      <c r="F7" s="2">
         <v>45191</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1271,11 +1357,14 @@
       <c r="D8" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" t="s">
+        <v>215</v>
+      </c>
+      <c r="F8" s="2">
         <v>45233</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1288,11 +1377,14 @@
       <c r="D9" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" t="s">
+        <v>216</v>
+      </c>
+      <c r="F9" s="2">
         <v>45317</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1305,11 +1397,14 @@
       <c r="D10" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" t="s">
+        <v>217</v>
+      </c>
+      <c r="F10" s="2">
         <v>45373</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1322,11 +1417,14 @@
       <c r="D11" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" t="s">
+        <v>218</v>
+      </c>
+      <c r="F11" s="2">
         <v>45436</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1339,11 +1437,14 @@
       <c r="D12" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" t="s">
+        <v>219</v>
+      </c>
+      <c r="F12" s="2">
         <v>45506</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1356,11 +1457,14 @@
       <c r="D13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" t="s">
+        <v>220</v>
+      </c>
+      <c r="F13" s="2">
         <v>45548</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1373,11 +1477,14 @@
       <c r="D14" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" t="s">
+        <v>221</v>
+      </c>
+      <c r="F14" s="2">
         <v>45604</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1390,11 +1497,14 @@
       <c r="D15" t="s">
         <v>73</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" t="s">
+        <v>222</v>
+      </c>
+      <c r="F15" s="2">
         <v>45674</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1407,11 +1517,14 @@
       <c r="D16" t="s">
         <v>74</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" t="s">
+        <v>223</v>
+      </c>
+      <c r="F16" s="2">
         <v>45744</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1424,11 +1537,14 @@
       <c r="D17" t="s">
         <v>75</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" t="s">
+        <v>224</v>
+      </c>
+      <c r="F17" s="2">
         <v>45807</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1441,11 +1557,14 @@
       <c r="D18" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" t="s">
+        <v>225</v>
+      </c>
+      <c r="F18" s="2">
         <v>45856</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1458,11 +1577,14 @@
       <c r="D19" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" t="s">
+        <v>226</v>
+      </c>
+      <c r="F19" s="2">
         <v>45856</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1475,11 +1597,11 @@
       <c r="D20" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="2">
+      <c r="F20" s="2">
         <v>45925</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1492,11 +1614,11 @@
       <c r="D21" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="2">
+      <c r="F21" s="2">
         <v>45925</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1509,11 +1631,14 @@
       <c r="D22" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" t="s">
+        <v>227</v>
+      </c>
+      <c r="F22" s="2">
         <v>45926</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1526,11 +1651,14 @@
       <c r="D23" t="s">
         <v>40</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" t="s">
+        <v>228</v>
+      </c>
+      <c r="F23" s="2">
         <v>45975</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1543,11 +1671,14 @@
       <c r="D24" t="s">
         <v>39</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" t="s">
+        <v>229</v>
+      </c>
+      <c r="F24" s="2">
         <v>46052</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1560,11 +1691,14 @@
       <c r="D25" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" t="s">
+        <v>230</v>
+      </c>
+      <c r="F25" s="2">
         <v>46108</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1577,11 +1711,14 @@
       <c r="D26" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" t="s">
+        <v>231</v>
+      </c>
+      <c r="F26" s="2">
         <v>46164</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1594,13 +1731,16 @@
       <c r="D27" t="s">
         <v>28</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" t="s">
+        <v>232</v>
+      </c>
+      <c r="F27" s="2">
         <v>46220</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:E27">
-    <sortCondition ref="E2:E27"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:F27">
+    <sortCondition ref="F2:F27"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add tournament metadata and support expanded card identifiers
</commit_message>
<xml_diff>
--- a/metadata/metadata.xlsx
+++ b/metadata/metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madis\Documents\pokemon_scraper\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0DB85E6-0613-4051-92D8-8FF68D36BB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F3918E-0908-4584-A1F6-9C259773C432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-2460" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-2460" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tournaments" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="256">
   <si>
     <t>tournament_id</t>
   </si>
@@ -729,6 +729,75 @@
   </si>
   <si>
     <t>pbl.png</t>
+  </si>
+  <si>
+    <t>30C</t>
+  </si>
+  <si>
+    <t>30th Celebration</t>
+  </si>
+  <si>
+    <t>Worlds 2026</t>
+  </si>
+  <si>
+    <t>Worlds</t>
+  </si>
+  <si>
+    <t>San Francisco</t>
+  </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>Baltimore</t>
+  </si>
+  <si>
+    <t>Regional</t>
+  </si>
+  <si>
+    <t>Maryland</t>
+  </si>
+  <si>
+    <t>Brisbane</t>
+  </si>
+  <si>
+    <t>Frankfurt</t>
+  </si>
+  <si>
+    <t>Recife</t>
+  </si>
+  <si>
+    <t>AUS</t>
+  </si>
+  <si>
+    <t>GER</t>
+  </si>
+  <si>
+    <t>BRA</t>
+  </si>
+  <si>
+    <t>Queensland</t>
+  </si>
+  <si>
+    <t>Hesse</t>
+  </si>
+  <si>
+    <t>Pernambuco</t>
+  </si>
+  <si>
+    <t>RE001-a2hqIrDZOyenzQ</t>
+  </si>
+  <si>
+    <t>FR001-qWsas6LjddfVxo</t>
+  </si>
+  <si>
+    <t>BR001-5YdU57MmWxTxaY</t>
+  </si>
+  <si>
+    <t>BA001-nEN1xl5ZJLGtFk</t>
+  </si>
+  <si>
+    <t>WCS01wI9lfI55wHtvrdy</t>
   </si>
 </sst>
 </file>
@@ -1058,21 +1127,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1190,6 +1260,196 @@
       </c>
       <c r="L3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B4" t="s">
+        <v>235</v>
+      </c>
+      <c r="C4">
+        <v>2026</v>
+      </c>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>236</v>
+      </c>
+      <c r="G4" t="s">
+        <v>237</v>
+      </c>
+      <c r="H4" t="s">
+        <v>238</v>
+      </c>
+      <c r="I4" t="s">
+        <v>83</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46262</v>
+      </c>
+      <c r="K4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C5">
+        <v>2026</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>240</v>
+      </c>
+      <c r="G5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H5" t="s">
+        <v>241</v>
+      </c>
+      <c r="I5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J5" s="2">
+        <v>46284</v>
+      </c>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6">
+        <v>2026</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>240</v>
+      </c>
+      <c r="G6" t="s">
+        <v>242</v>
+      </c>
+      <c r="H6" t="s">
+        <v>248</v>
+      </c>
+      <c r="I6" t="s">
+        <v>245</v>
+      </c>
+      <c r="J6" s="2">
+        <v>46291</v>
+      </c>
+      <c r="K6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C7">
+        <v>2026</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>240</v>
+      </c>
+      <c r="G7" t="s">
+        <v>243</v>
+      </c>
+      <c r="H7" t="s">
+        <v>249</v>
+      </c>
+      <c r="I7" t="s">
+        <v>246</v>
+      </c>
+      <c r="J7" s="2">
+        <v>46291</v>
+      </c>
+      <c r="K7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>251</v>
+      </c>
+      <c r="B8" t="s">
+        <v>244</v>
+      </c>
+      <c r="C8">
+        <v>2026</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>240</v>
+      </c>
+      <c r="G8" t="s">
+        <v>244</v>
+      </c>
+      <c r="H8" t="s">
+        <v>250</v>
+      </c>
+      <c r="I8" t="s">
+        <v>247</v>
+      </c>
+      <c r="J8" s="2">
+        <v>46298</v>
+      </c>
+      <c r="K8" t="s">
+        <v>20</v>
+      </c>
+      <c r="L8" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -1200,7 +1460,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0D6416A-2744-408B-ACBE-6C19FD322B6D}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
@@ -1736,6 +1996,23 @@
       </c>
       <c r="F27" s="2">
         <v>46220</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" t="s">
+        <v>233</v>
+      </c>
+      <c r="D28" t="s">
+        <v>234</v>
+      </c>
+      <c r="F28" s="2">
+        <v>46281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add archetype representative card contact sheet
</commit_message>
<xml_diff>
--- a/metadata/metadata.xlsx
+++ b/metadata/metadata.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madis\Documents\pokemon_scraper\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F3918E-0908-4584-A1F6-9C259773C432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F873A2EF-CC52-45F0-8E2C-43D3DEE09BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-2460" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tournaments" sheetId="1" r:id="rId1"/>
     <sheet name="sets" sheetId="4" r:id="rId2"/>
     <sheet name="archetypes" sheetId="5" r:id="rId3"/>
+    <sheet name="archetype_cards" sheetId="8" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">archetypes!$A$1:$F$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">archetype_cards!$A$1:$D$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">archetypes!$A$1:$F$122</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="370">
   <si>
     <t>tournament_id</t>
   </si>
@@ -434,9 +436,6 @@
     <t>Mega Starmie ex</t>
   </si>
   <si>
-    <t>Mega Frosslass ex</t>
-  </si>
-  <si>
     <t>Mega Greninja</t>
   </si>
   <si>
@@ -798,6 +797,351 @@
   </si>
   <si>
     <t>WCS01wI9lfI55wHtvrdy</t>
+  </si>
+  <si>
+    <t>representative_card_id</t>
+  </si>
+  <si>
+    <t>representative_card_id_2</t>
+  </si>
+  <si>
+    <t>Mega Excadrill</t>
+  </si>
+  <si>
+    <t>Hide 'n' Sneak</t>
+  </si>
+  <si>
+    <t>Dhelmise</t>
+  </si>
+  <si>
+    <t>Dipplin</t>
+  </si>
+  <si>
+    <t>Seaking</t>
+  </si>
+  <si>
+    <t>Mega Chandelure</t>
+  </si>
+  <si>
+    <t>Mega Chandelure ex</t>
+  </si>
+  <si>
+    <t>Mega Darkrai</t>
+  </si>
+  <si>
+    <t>Mega Darkrai ex</t>
+  </si>
+  <si>
+    <t>Toucannon</t>
+  </si>
+  <si>
+    <t>Mew</t>
+  </si>
+  <si>
+    <t>Mew ex</t>
+  </si>
+  <si>
+    <t>Louisville</t>
+  </si>
+  <si>
+    <t>Kentucky</t>
+  </si>
+  <si>
+    <t>LO001-piALjQswPD3x0J</t>
+  </si>
+  <si>
+    <t>Nice</t>
+  </si>
+  <si>
+    <t>Puebla</t>
+  </si>
+  <si>
+    <t>Gdansk</t>
+  </si>
+  <si>
+    <t>LAIC 2027</t>
+  </si>
+  <si>
+    <t>Stuttgart</t>
+  </si>
+  <si>
+    <t>Las Vegas</t>
+  </si>
+  <si>
+    <t>FRA</t>
+  </si>
+  <si>
+    <t>Nevada</t>
+  </si>
+  <si>
+    <t>NC001-2OXFgm7aAOcHKh</t>
+  </si>
+  <si>
+    <t>PB001-35rH2yUmy8TR3M</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>POL</t>
+  </si>
+  <si>
+    <t>GD001-Hoo7UUNiVvyRG4</t>
+  </si>
+  <si>
+    <t>Sao Paulo</t>
+  </si>
+  <si>
+    <t>LA001-jHlXupaysix7HO</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>SG001-9JttihqdIjqHBR</t>
+  </si>
+  <si>
+    <t>LV001-Wwe32kM2VwJ94M</t>
+  </si>
+  <si>
+    <t>Mega Froslass ex</t>
+  </si>
+  <si>
+    <t>Froslass</t>
+  </si>
+  <si>
+    <t>Mega Excadrill ex</t>
+  </si>
+  <si>
+    <t>me01-056</t>
+  </si>
+  <si>
+    <t>sv08-130</t>
+  </si>
+  <si>
+    <t>me02.5-084</t>
+  </si>
+  <si>
+    <t>me04-003</t>
+  </si>
+  <si>
+    <t>sv09-024</t>
+  </si>
+  <si>
+    <t>sv06-134</t>
+  </si>
+  <si>
+    <t>sv06.5-025</t>
+  </si>
+  <si>
+    <t>sv07-119</t>
+  </si>
+  <si>
+    <t>sv05-069</t>
+  </si>
+  <si>
+    <t>sv08-036</t>
+  </si>
+  <si>
+    <t>me04-073</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sv10-012 </t>
+  </si>
+  <si>
+    <t>me02.5-111</t>
+  </si>
+  <si>
+    <t>me03-012</t>
+  </si>
+  <si>
+    <t>me05-039</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> sv06-018</t>
+  </si>
+  <si>
+    <t>me03-057</t>
+  </si>
+  <si>
+    <t>sv06-130</t>
+  </si>
+  <si>
+    <t>sv05-129</t>
+  </si>
+  <si>
+    <t>sv06.5-020</t>
+  </si>
+  <si>
+    <t>sv10-034</t>
+  </si>
+  <si>
+    <t>sv05-041</t>
+  </si>
+  <si>
+    <t>sv08.5-014</t>
+  </si>
+  <si>
+    <t>me02.5-096</t>
+  </si>
+  <si>
+    <t>sv10-023</t>
+  </si>
+  <si>
+    <t>sv07-014</t>
+  </si>
+  <si>
+    <t>sv08-119</t>
+  </si>
+  <si>
+    <t>me02.5-070</t>
+  </si>
+  <si>
+    <t>sv07-050</t>
+  </si>
+  <si>
+    <t>me02.5-076</t>
+  </si>
+  <si>
+    <t>me02.5-287</t>
+  </si>
+  <si>
+    <t>me01-036</t>
+  </si>
+  <si>
+    <t>me01-08</t>
+  </si>
+  <si>
+    <t>me05-038</t>
+  </si>
+  <si>
+    <t>me05-048</t>
+  </si>
+  <si>
+    <t>me02.5-267</t>
+  </si>
+  <si>
+    <t>me02.5-152</t>
+  </si>
+  <si>
+    <t>me04-022</t>
+  </si>
+  <si>
+    <t>me01-10</t>
+  </si>
+  <si>
+    <t>me02-08</t>
+  </si>
+  <si>
+    <t>me01-07</t>
+  </si>
+  <si>
+    <t>me01-050</t>
+  </si>
+  <si>
+    <t>me02-061</t>
+  </si>
+  <si>
+    <t>me03-021</t>
+  </si>
+  <si>
+    <t>me03-047</t>
+  </si>
+  <si>
+    <t>me01-01</t>
+  </si>
+  <si>
+    <t>me03-062</t>
+  </si>
+  <si>
+    <t>me04-061</t>
+  </si>
+  <si>
+    <t>sv05-114</t>
+  </si>
+  <si>
+    <t>sv03.5-151</t>
+  </si>
+  <si>
+    <t>sv09-09</t>
+  </si>
+  <si>
+    <t>sv07-115</t>
+  </si>
+  <si>
+    <t>sv10-003</t>
+  </si>
+  <si>
+    <t>sv06-064</t>
+  </si>
+  <si>
+    <t>me05-068</t>
+  </si>
+  <si>
+    <t>me02-06</t>
+  </si>
+  <si>
+    <t>sv06-015</t>
+  </si>
+  <si>
+    <t>sv10-020</t>
+  </si>
+  <si>
+    <t>sv10-081</t>
+  </si>
+  <si>
+    <t>me02.5-127</t>
+  </si>
+  <si>
+    <t>sv06-025</t>
+  </si>
+  <si>
+    <t>sv10-145</t>
+  </si>
+  <si>
+    <t>sv07-058</t>
+  </si>
+  <si>
+    <t>sv08.5-019</t>
+  </si>
+  <si>
+    <t>sv05-123</t>
+  </si>
+  <si>
+    <t>sv06-06</t>
+  </si>
+  <si>
+    <t>sv08.5-04</t>
+  </si>
+  <si>
+    <t>sv06-111</t>
+  </si>
+  <si>
+    <t>sv06-053</t>
+  </si>
+  <si>
+    <t>sv06-106</t>
+  </si>
+  <si>
+    <t>sv06.5-047</t>
+  </si>
+  <si>
+    <t>sv09-151</t>
+  </si>
+  <si>
+    <t>me05-06</t>
+  </si>
+  <si>
+    <t>me01-003</t>
+  </si>
+  <si>
+    <t>sv08-057</t>
+  </si>
+  <si>
+    <t>sv04-066</t>
   </si>
 </sst>
 </file>
@@ -1127,10 +1471,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -1139,7 +1483,7 @@
     <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
@@ -1264,10 +1608,10 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C4">
         <v>2026</v>
@@ -1279,13 +1623,13 @@
         <v>13</v>
       </c>
       <c r="F4" t="s">
+        <v>235</v>
+      </c>
+      <c r="G4" t="s">
         <v>236</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>237</v>
-      </c>
-      <c r="H4" t="s">
-        <v>238</v>
       </c>
       <c r="I4" t="s">
         <v>83</v>
@@ -1302,13 +1646,13 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D5" t="s">
         <v>18</v>
@@ -1317,13 +1661,13 @@
         <v>13</v>
       </c>
       <c r="F5" t="s">
+        <v>239</v>
+      </c>
+      <c r="G5" t="s">
+        <v>238</v>
+      </c>
+      <c r="H5" t="s">
         <v>240</v>
-      </c>
-      <c r="G5" t="s">
-        <v>239</v>
-      </c>
-      <c r="H5" t="s">
-        <v>241</v>
       </c>
       <c r="I5" t="s">
         <v>83</v>
@@ -1340,13 +1684,13 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C6">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
@@ -1355,16 +1699,16 @@
         <v>13</v>
       </c>
       <c r="F6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J6" s="2">
         <v>46291</v>
@@ -1373,18 +1717,18 @@
         <v>20</v>
       </c>
       <c r="L6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C7">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -1393,16 +1737,16 @@
         <v>13</v>
       </c>
       <c r="F7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J7" s="2">
         <v>46291</v>
@@ -1411,18 +1755,18 @@
         <v>20</v>
       </c>
       <c r="L7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C8">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D8" t="s">
         <v>18</v>
@@ -1431,16 +1775,16 @@
         <v>13</v>
       </c>
       <c r="F8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J8" s="2">
         <v>46298</v>
@@ -1449,7 +1793,243 @@
         <v>20</v>
       </c>
       <c r="L8" t="s">
-        <v>233</v>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>271</v>
+      </c>
+      <c r="B9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C9">
+        <v>2027</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
+        <v>239</v>
+      </c>
+      <c r="G9" t="s">
+        <v>269</v>
+      </c>
+      <c r="H9" t="s">
+        <v>270</v>
+      </c>
+      <c r="I9" t="s">
+        <v>83</v>
+      </c>
+      <c r="J9" s="2">
+        <v>46304</v>
+      </c>
+      <c r="K9" t="s">
+        <v>20</v>
+      </c>
+      <c r="L9" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>280</v>
+      </c>
+      <c r="B10" t="s">
+        <v>272</v>
+      </c>
+      <c r="C10">
+        <v>2027</v>
+      </c>
+      <c r="D10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
+        <v>239</v>
+      </c>
+      <c r="G10" t="s">
+        <v>272</v>
+      </c>
+      <c r="H10" t="s">
+        <v>283</v>
+      </c>
+      <c r="I10" t="s">
+        <v>278</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46312</v>
+      </c>
+      <c r="K10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>281</v>
+      </c>
+      <c r="B11" t="s">
+        <v>273</v>
+      </c>
+      <c r="C11">
+        <v>2027</v>
+      </c>
+      <c r="D11" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
+        <v>239</v>
+      </c>
+      <c r="G11" t="s">
+        <v>273</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46319</v>
+      </c>
+      <c r="K11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>285</v>
+      </c>
+      <c r="B12" t="s">
+        <v>274</v>
+      </c>
+      <c r="C12">
+        <v>2027</v>
+      </c>
+      <c r="D12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>239</v>
+      </c>
+      <c r="G12" t="s">
+        <v>274</v>
+      </c>
+      <c r="H12" t="s">
+        <v>282</v>
+      </c>
+      <c r="I12" t="s">
+        <v>284</v>
+      </c>
+      <c r="J12" s="2">
+        <v>46326</v>
+      </c>
+      <c r="K12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>287</v>
+      </c>
+      <c r="B13" t="s">
+        <v>275</v>
+      </c>
+      <c r="C13">
+        <v>2027</v>
+      </c>
+      <c r="D13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" t="s">
+        <v>286</v>
+      </c>
+      <c r="J13" s="2">
+        <v>46346</v>
+      </c>
+      <c r="K13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>289</v>
+      </c>
+      <c r="B14" t="s">
+        <v>276</v>
+      </c>
+      <c r="C14">
+        <v>2027</v>
+      </c>
+      <c r="D14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>239</v>
+      </c>
+      <c r="G14" t="s">
+        <v>276</v>
+      </c>
+      <c r="H14" t="s">
+        <v>288</v>
+      </c>
+      <c r="I14" t="s">
+        <v>245</v>
+      </c>
+      <c r="J14" s="2">
+        <v>46354</v>
+      </c>
+      <c r="K14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>290</v>
+      </c>
+      <c r="B15" t="s">
+        <v>277</v>
+      </c>
+      <c r="C15">
+        <v>2027</v>
+      </c>
+      <c r="D15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>239</v>
+      </c>
+      <c r="G15" t="s">
+        <v>277</v>
+      </c>
+      <c r="H15" t="s">
+        <v>279</v>
+      </c>
+      <c r="I15" t="s">
+        <v>83</v>
+      </c>
+      <c r="J15" s="2">
+        <v>46360</v>
+      </c>
+      <c r="K15" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1484,7 +2064,7 @@
         <v>24</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>25</v>
@@ -1538,7 +2118,7 @@
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F4" s="2">
         <v>45016</v>
@@ -1558,7 +2138,7 @@
         <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F5" s="2">
         <v>45086</v>
@@ -1578,7 +2158,7 @@
         <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F6" s="2">
         <v>45149</v>
@@ -1598,7 +2178,7 @@
         <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F7" s="2">
         <v>45191</v>
@@ -1618,7 +2198,7 @@
         <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F8" s="2">
         <v>45233</v>
@@ -1638,7 +2218,7 @@
         <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F9" s="2">
         <v>45317</v>
@@ -1658,7 +2238,7 @@
         <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F10" s="2">
         <v>45373</v>
@@ -1678,7 +2258,7 @@
         <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F11" s="2">
         <v>45436</v>
@@ -1698,7 +2278,7 @@
         <v>70</v>
       </c>
       <c r="E12" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F12" s="2">
         <v>45506</v>
@@ -1718,7 +2298,7 @@
         <v>71</v>
       </c>
       <c r="E13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F13" s="2">
         <v>45548</v>
@@ -1738,7 +2318,7 @@
         <v>72</v>
       </c>
       <c r="E14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F14" s="2">
         <v>45604</v>
@@ -1758,7 +2338,7 @@
         <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F15" s="2">
         <v>45674</v>
@@ -1778,7 +2358,7 @@
         <v>74</v>
       </c>
       <c r="E16" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F16" s="2">
         <v>45744</v>
@@ -1798,7 +2378,7 @@
         <v>75</v>
       </c>
       <c r="E17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F17" s="2">
         <v>45807</v>
@@ -1818,7 +2398,7 @@
         <v>77</v>
       </c>
       <c r="E18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F18" s="2">
         <v>45856</v>
@@ -1838,7 +2418,7 @@
         <v>76</v>
       </c>
       <c r="E19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F19" s="2">
         <v>45856</v>
@@ -1892,7 +2472,7 @@
         <v>41</v>
       </c>
       <c r="E22" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F22" s="2">
         <v>45926</v>
@@ -1912,7 +2492,7 @@
         <v>40</v>
       </c>
       <c r="E23" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F23" s="2">
         <v>45975</v>
@@ -1932,7 +2512,7 @@
         <v>39</v>
       </c>
       <c r="E24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F24" s="2">
         <v>46052</v>
@@ -1952,7 +2532,7 @@
         <v>38</v>
       </c>
       <c r="E25" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F25" s="2">
         <v>46108</v>
@@ -1972,7 +2552,7 @@
         <v>29</v>
       </c>
       <c r="E26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F26" s="2">
         <v>46164</v>
@@ -1992,7 +2572,7 @@
         <v>28</v>
       </c>
       <c r="E27" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F27" s="2">
         <v>46220</v>
@@ -2006,10 +2586,10 @@
         <v>27</v>
       </c>
       <c r="C28" t="s">
+        <v>232</v>
+      </c>
+      <c r="D28" t="s">
         <v>233</v>
-      </c>
-      <c r="D28" t="s">
-        <v>234</v>
       </c>
       <c r="F28" s="2">
         <v>46281</v>
@@ -2025,7 +2605,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}">
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -2203,7 +2783,7 @@
         <v>98</v>
       </c>
       <c r="C9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D9" t="s">
         <v>100</v>
@@ -2223,7 +2803,7 @@
         <v>101</v>
       </c>
       <c r="C10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
         <v>101</v>
@@ -2243,7 +2823,7 @@
         <v>102</v>
       </c>
       <c r="C11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D11" t="s">
         <v>102</v>
@@ -2263,7 +2843,7 @@
         <v>104</v>
       </c>
       <c r="C12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D12" t="s">
         <v>104</v>
@@ -2280,13 +2860,13 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>201</v>
+        <v>104</v>
       </c>
       <c r="C13" t="s">
-        <v>105</v>
+        <v>161</v>
       </c>
       <c r="D13" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
       <c r="E13" t="s">
         <v>95</v>
@@ -2297,56 +2877,56 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>201</v>
+        <v>104</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="E14" t="s">
         <v>95</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>201</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
         <v>95</v>
       </c>
       <c r="F15">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C16" t="s">
-        <v>162</v>
+        <v>105</v>
       </c>
       <c r="D16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E16" t="s">
         <v>95</v>
@@ -2357,16 +2937,16 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
+        <v>200</v>
+      </c>
+      <c r="C17" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" t="s">
         <v>201</v>
-      </c>
-      <c r="C17" t="s">
-        <v>162</v>
-      </c>
-      <c r="D17" t="s">
-        <v>202</v>
       </c>
       <c r="E17" t="s">
         <v>95</v>
@@ -2377,22 +2957,22 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C18" t="s">
-        <v>162</v>
+        <v>105</v>
       </c>
       <c r="D18" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E18" t="s">
-        <v>203</v>
+        <v>95</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -2400,139 +2980,139 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D19" t="s">
-        <v>113</v>
+        <v>158</v>
       </c>
       <c r="E19" t="s">
         <v>95</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>106</v>
+        <v>200</v>
       </c>
       <c r="C20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D20" t="s">
-        <v>109</v>
+        <v>201</v>
       </c>
       <c r="E20" t="s">
         <v>95</v>
       </c>
       <c r="F20">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>200</v>
       </c>
       <c r="C21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D21" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E21" t="s">
-        <v>95</v>
+        <v>202</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>106</v>
+        <v>200</v>
       </c>
       <c r="C22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D22" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E22" t="s">
         <v>95</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>200</v>
       </c>
       <c r="C23" t="s">
-        <v>162</v>
+        <v>267</v>
       </c>
       <c r="D23" t="s">
-        <v>113</v>
+        <v>158</v>
       </c>
       <c r="E23" t="s">
         <v>95</v>
       </c>
       <c r="F23">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="C24" t="s">
-        <v>162</v>
+        <v>267</v>
       </c>
       <c r="D24" t="s">
-        <v>115</v>
+        <v>201</v>
       </c>
       <c r="E24" t="s">
         <v>95</v>
       </c>
       <c r="F24">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>116</v>
+        <v>200</v>
       </c>
       <c r="C25" t="s">
-        <v>162</v>
+        <v>267</v>
       </c>
       <c r="D25" t="s">
-        <v>117</v>
+        <v>268</v>
       </c>
       <c r="E25" t="s">
         <v>95</v>
       </c>
       <c r="F25">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2540,19 +3120,19 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="C26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D26" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="E26" t="s">
         <v>95</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2560,19 +3140,19 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>182</v>
+        <v>106</v>
       </c>
       <c r="C27" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="D27" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="E27" t="s">
         <v>95</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2580,19 +3160,19 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>182</v>
+        <v>106</v>
       </c>
       <c r="C28" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="D28" t="s">
-        <v>185</v>
+        <v>111</v>
       </c>
       <c r="E28" t="s">
         <v>95</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2600,13 +3180,13 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D29" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="E29" t="s">
         <v>95</v>
@@ -2620,13 +3200,13 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D30" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E30" t="s">
         <v>95</v>
@@ -2640,13 +3220,13 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D31" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="E31" t="s">
         <v>95</v>
@@ -2660,13 +3240,13 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="C32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D32" t="s">
-        <v>125</v>
+        <v>260</v>
       </c>
       <c r="E32" t="s">
         <v>95</v>
@@ -2677,16 +3257,16 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C33" t="s">
-        <v>162</v>
+        <v>261</v>
       </c>
       <c r="D33" t="s">
-        <v>200</v>
+        <v>117</v>
       </c>
       <c r="E33" t="s">
         <v>95</v>
@@ -2697,22 +3277,22 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C34" t="s">
-        <v>162</v>
+        <v>261</v>
       </c>
       <c r="D34" t="s">
-        <v>126</v>
+        <v>261</v>
       </c>
       <c r="E34" t="s">
         <v>95</v>
       </c>
       <c r="F34">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2720,13 +3300,13 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="C35" t="s">
-        <v>90</v>
+        <v>161</v>
       </c>
       <c r="D35" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="E35" t="s">
         <v>95</v>
@@ -2740,79 +3320,79 @@
         <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>127</v>
+        <v>181</v>
       </c>
       <c r="C36" t="s">
-        <v>90</v>
+        <v>182</v>
       </c>
       <c r="D36" t="s">
-        <v>90</v>
+        <v>163</v>
       </c>
       <c r="E36" t="s">
         <v>95</v>
       </c>
       <c r="F36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>127</v>
+        <v>181</v>
       </c>
       <c r="C37" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="D37" t="s">
-        <v>128</v>
+        <v>184</v>
       </c>
       <c r="E37" t="s">
         <v>95</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D38" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="E38" t="s">
         <v>95</v>
       </c>
       <c r="F38">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C39" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D39" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="E39" t="s">
         <v>95</v>
       </c>
       <c r="F39">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2820,19 +3400,19 @@
         <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="C40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D40" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="E40" t="s">
         <v>95</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2840,19 +3420,19 @@
         <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>163</v>
+        <v>124</v>
       </c>
       <c r="C41" t="s">
-        <v>132</v>
+        <v>161</v>
       </c>
       <c r="D41" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="E41" t="s">
         <v>95</v>
       </c>
       <c r="F41">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2860,73 +3440,73 @@
         <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>163</v>
+        <v>257</v>
       </c>
       <c r="C42" t="s">
-        <v>132</v>
+        <v>161</v>
       </c>
       <c r="D42" t="s">
-        <v>134</v>
+        <v>293</v>
       </c>
       <c r="E42" t="s">
         <v>95</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>163</v>
+        <v>126</v>
       </c>
       <c r="C43" t="s">
-        <v>90</v>
+        <v>161</v>
       </c>
       <c r="D43" t="s">
-        <v>133</v>
+        <v>199</v>
       </c>
       <c r="E43" t="s">
         <v>95</v>
       </c>
       <c r="F43">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>163</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>90</v>
+        <v>161</v>
       </c>
       <c r="D44" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="E44" t="s">
         <v>95</v>
       </c>
       <c r="F44">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="C45" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D45" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E45" t="s">
         <v>95</v>
@@ -2940,33 +3520,33 @@
         <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C46" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D46" t="s">
-        <v>136</v>
+        <v>90</v>
       </c>
       <c r="E46" t="s">
         <v>95</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B47" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="D47" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="E47" t="s">
         <v>95</v>
@@ -2977,16 +3557,16 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B48" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C48" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="D48" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="E48" t="s">
         <v>95</v>
@@ -2997,16 +3577,16 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B49" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C49" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="D49" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="E49" t="s">
         <v>95</v>
@@ -3017,16 +3597,16 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B50" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C50" t="s">
-        <v>103</v>
+        <v>161</v>
       </c>
       <c r="D50" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="E50" t="s">
         <v>95</v>
@@ -3037,16 +3617,16 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C51" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="D51" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E51" t="s">
         <v>95</v>
@@ -3057,36 +3637,36 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C52" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="D52" t="s">
-        <v>107</v>
+        <v>291</v>
       </c>
       <c r="E52" t="s">
         <v>95</v>
       </c>
       <c r="F52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B53" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C53" t="s">
-        <v>198</v>
+        <v>90</v>
       </c>
       <c r="D53" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="E53" t="s">
         <v>95</v>
@@ -3097,22 +3677,22 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C54" t="s">
-        <v>198</v>
+        <v>90</v>
       </c>
       <c r="D54" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="E54" t="s">
         <v>95</v>
       </c>
       <c r="F54">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -3120,13 +3700,13 @@
         <v>30</v>
       </c>
       <c r="B55" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C55" t="s">
-        <v>198</v>
+        <v>161</v>
       </c>
       <c r="D55" t="s">
-        <v>199</v>
+        <v>133</v>
       </c>
       <c r="E55" t="s">
         <v>95</v>
@@ -3137,16 +3717,16 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="B56" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D56" t="s">
-        <v>109</v>
+        <v>135</v>
       </c>
       <c r="E56" t="s">
         <v>95</v>
@@ -3157,16 +3737,16 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="B57" t="s">
+        <v>136</v>
+      </c>
+      <c r="C57" t="s">
         <v>137</v>
       </c>
-      <c r="C57" t="s">
-        <v>162</v>
-      </c>
       <c r="D57" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="E57" t="s">
         <v>95</v>
@@ -3180,13 +3760,13 @@
         <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C58" t="s">
-        <v>162</v>
+        <v>137</v>
       </c>
       <c r="D58" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E58" t="s">
         <v>95</v>
@@ -3200,13 +3780,13 @@
         <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C59" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D59" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E59" t="s">
         <v>95</v>
@@ -3217,16 +3797,16 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B60" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C60" t="s">
-        <v>143</v>
+        <v>103</v>
       </c>
       <c r="D60" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="E60" t="s">
         <v>95</v>
@@ -3240,13 +3820,13 @@
         <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C61" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D61" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E61" t="s">
         <v>95</v>
@@ -3260,13 +3840,13 @@
         <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C62" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D62" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E62" t="s">
         <v>95</v>
@@ -3280,13 +3860,13 @@
         <v>30</v>
       </c>
       <c r="B63" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C63" t="s">
-        <v>162</v>
+        <v>197</v>
       </c>
       <c r="D63" t="s">
-        <v>144</v>
+        <v>109</v>
       </c>
       <c r="E63" t="s">
         <v>95</v>
@@ -3297,16 +3877,16 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B64" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C64" t="s">
-        <v>162</v>
+        <v>197</v>
       </c>
       <c r="D64" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="E64" t="s">
         <v>95</v>
@@ -3317,16 +3897,16 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B65" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="C65" t="s">
-        <v>162</v>
+        <v>197</v>
       </c>
       <c r="D65" t="s">
-        <v>147</v>
+        <v>198</v>
       </c>
       <c r="E65" t="s">
         <v>95</v>
@@ -3337,16 +3917,16 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B66" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="C66" t="s">
-        <v>90</v>
+        <v>161</v>
       </c>
       <c r="D66" t="s">
-        <v>150</v>
+        <v>109</v>
       </c>
       <c r="E66" t="s">
         <v>95</v>
@@ -3357,16 +3937,16 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B67" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>161</v>
       </c>
       <c r="D67" t="s">
-        <v>90</v>
+        <v>138</v>
       </c>
       <c r="E67" t="s">
         <v>95</v>
@@ -3377,16 +3957,16 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B68" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="C68" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D68" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E68" t="s">
         <v>95</v>
@@ -3400,19 +3980,19 @@
         <v>10</v>
       </c>
       <c r="B69" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C69" t="s">
-        <v>162</v>
+        <v>142</v>
       </c>
       <c r="D69" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="E69" t="s">
         <v>95</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -3420,13 +4000,13 @@
         <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C70" t="s">
-        <v>162</v>
+        <v>142</v>
       </c>
       <c r="D70" t="s">
-        <v>152</v>
+        <v>100</v>
       </c>
       <c r="E70" t="s">
         <v>95</v>
@@ -3437,16 +4017,16 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B71" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C71" t="s">
-        <v>162</v>
+        <v>97</v>
       </c>
       <c r="D71" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="E71" t="s">
         <v>95</v>
@@ -3457,16 +4037,16 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B72" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C72" t="s">
-        <v>162</v>
+        <v>97</v>
       </c>
       <c r="D72" t="s">
-        <v>156</v>
+        <v>97</v>
       </c>
       <c r="E72" t="s">
         <v>95</v>
@@ -3477,16 +4057,16 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B73" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C73" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D73" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="E73" t="s">
         <v>95</v>
@@ -3500,13 +4080,13 @@
         <v>10</v>
       </c>
       <c r="B74" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="C74" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D74" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="E74" t="s">
         <v>95</v>
@@ -3520,13 +4100,13 @@
         <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="C75" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D75" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
       <c r="E75" t="s">
         <v>95</v>
@@ -3540,19 +4120,19 @@
         <v>10</v>
       </c>
       <c r="B76" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="C76" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E76" t="s">
         <v>95</v>
       </c>
       <c r="F76">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -3560,33 +4140,33 @@
         <v>10</v>
       </c>
       <c r="B77" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="C77" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>165</v>
+        <v>90</v>
       </c>
       <c r="E77" t="s">
         <v>95</v>
       </c>
       <c r="F77">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B78" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="C78" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D78" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="E78" t="s">
         <v>95</v>
@@ -3600,19 +4180,19 @@
         <v>10</v>
       </c>
       <c r="B79" t="s">
-        <v>187</v>
+        <v>150</v>
       </c>
       <c r="C79" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D79" t="s">
-        <v>186</v>
+        <v>110</v>
       </c>
       <c r="E79" t="s">
         <v>95</v>
       </c>
       <c r="F79">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -3620,19 +4200,19 @@
         <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="C80" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D80" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="E80" t="s">
         <v>95</v>
       </c>
       <c r="F80">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -3640,13 +4220,13 @@
         <v>10</v>
       </c>
       <c r="B81" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="C81" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D81" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="E81" t="s">
         <v>95</v>
@@ -3660,13 +4240,13 @@
         <v>10</v>
       </c>
       <c r="B82" t="s">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="C82" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D82" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="E82" t="s">
         <v>95</v>
@@ -3680,13 +4260,13 @@
         <v>10</v>
       </c>
       <c r="B83" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="C83" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D83" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="E83" t="s">
         <v>95</v>
@@ -3700,13 +4280,13 @@
         <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="C84" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D84" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="E84" t="s">
         <v>95</v>
@@ -3720,13 +4300,13 @@
         <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="C85" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D85" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
       <c r="E85" t="s">
         <v>95</v>
@@ -3740,19 +4320,19 @@
         <v>10</v>
       </c>
       <c r="B86" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="C86" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D86" t="s">
-        <v>179</v>
+        <v>156</v>
       </c>
       <c r="E86" t="s">
         <v>95</v>
       </c>
       <c r="F86">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3760,19 +4340,19 @@
         <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="C87" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D87" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="E87" t="s">
         <v>95</v>
       </c>
       <c r="F87">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -3780,13 +4360,13 @@
         <v>10</v>
       </c>
       <c r="B88" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="C88" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D88" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
       <c r="E88" t="s">
         <v>95</v>
@@ -3800,13 +4380,13 @@
         <v>10</v>
       </c>
       <c r="B89" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C89" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D89" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E89" t="s">
         <v>95</v>
@@ -3820,19 +4400,19 @@
         <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="C90" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D90" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="E90" t="s">
         <v>95</v>
       </c>
       <c r="F90">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -3840,13 +4420,13 @@
         <v>10</v>
       </c>
       <c r="B91" t="s">
-        <v>193</v>
+        <v>167</v>
       </c>
       <c r="C91" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D91" t="s">
-        <v>194</v>
+        <v>168</v>
       </c>
       <c r="E91" t="s">
         <v>95</v>
@@ -3860,19 +4440,19 @@
         <v>10</v>
       </c>
       <c r="B92" t="s">
-        <v>195</v>
+        <v>169</v>
       </c>
       <c r="C92" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D92" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
       <c r="E92" t="s">
         <v>95</v>
       </c>
       <c r="F92">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3880,13 +4460,13 @@
         <v>10</v>
       </c>
       <c r="B93" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="C93" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D93" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="E93" t="s">
         <v>95</v>
@@ -3900,13 +4480,13 @@
         <v>10</v>
       </c>
       <c r="B94" t="s">
-        <v>197</v>
+        <v>173</v>
       </c>
       <c r="C94" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D94" t="s">
-        <v>197</v>
+        <v>174</v>
       </c>
       <c r="E94" t="s">
         <v>95</v>
@@ -3920,13 +4500,13 @@
         <v>10</v>
       </c>
       <c r="B95" t="s">
-        <v>105</v>
+        <v>175</v>
       </c>
       <c r="C95" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="D95" t="s">
-        <v>108</v>
+        <v>176</v>
       </c>
       <c r="E95" t="s">
         <v>95</v>
@@ -3940,13 +4520,13 @@
         <v>10</v>
       </c>
       <c r="B96" t="s">
-        <v>105</v>
+        <v>177</v>
       </c>
       <c r="C96" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="D96" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
       <c r="E96" t="s">
         <v>95</v>
@@ -3957,16 +4537,16 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B97" t="s">
-        <v>105</v>
+        <v>179</v>
       </c>
       <c r="C97" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D97" t="s">
-        <v>108</v>
+        <v>180</v>
       </c>
       <c r="E97" t="s">
         <v>95</v>
@@ -3977,22 +4557,22 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>105</v>
+        <v>187</v>
       </c>
       <c r="C98" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D98" t="s">
-        <v>109</v>
+        <v>188</v>
       </c>
       <c r="E98" t="s">
         <v>95</v>
       </c>
       <c r="F98">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -4000,13 +4580,13 @@
         <v>10</v>
       </c>
       <c r="B99" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C99" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D99" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="E99" t="s">
         <v>95</v>
@@ -4020,13 +4600,13 @@
         <v>10</v>
       </c>
       <c r="B100" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C100" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D100" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="E100" t="s">
         <v>95</v>
@@ -4040,13 +4620,13 @@
         <v>10</v>
       </c>
       <c r="B101" t="s">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="C101" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D101" t="s">
-        <v>89</v>
+        <v>193</v>
       </c>
       <c r="E101" t="s">
         <v>95</v>
@@ -4060,39 +4640,39 @@
         <v>10</v>
       </c>
       <c r="B102" t="s">
-        <v>96</v>
+        <v>194</v>
       </c>
       <c r="C102" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D102" t="s">
-        <v>100</v>
+        <v>195</v>
       </c>
       <c r="E102" t="s">
         <v>95</v>
       </c>
       <c r="F102">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B103" t="s">
-        <v>96</v>
+        <v>194</v>
       </c>
       <c r="C103" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D103" t="s">
-        <v>89</v>
+        <v>151</v>
       </c>
       <c r="E103" t="s">
         <v>95</v>
       </c>
       <c r="F103">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -4100,13 +4680,13 @@
         <v>10</v>
       </c>
       <c r="B104" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="C104" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D104" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="E104" t="s">
         <v>95</v>
@@ -4120,13 +4700,13 @@
         <v>10</v>
       </c>
       <c r="B105" t="s">
-        <v>138</v>
+        <v>105</v>
       </c>
       <c r="C105" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="D105" t="s">
-        <v>140</v>
+        <v>108</v>
       </c>
       <c r="E105" t="s">
         <v>95</v>
@@ -4140,13 +4720,13 @@
         <v>10</v>
       </c>
       <c r="B106" t="s">
-        <v>138</v>
+        <v>105</v>
       </c>
       <c r="C106" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="D106" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="E106" t="s">
         <v>95</v>
@@ -4160,13 +4740,13 @@
         <v>20</v>
       </c>
       <c r="B107" t="s">
-        <v>138</v>
+        <v>105</v>
       </c>
       <c r="C107" t="s">
-        <v>90</v>
+        <v>161</v>
       </c>
       <c r="D107" t="s">
-        <v>140</v>
+        <v>108</v>
       </c>
       <c r="E107" t="s">
         <v>95</v>
@@ -4180,23 +4760,1330 @@
         <v>20</v>
       </c>
       <c r="B108" t="s">
-        <v>138</v>
+        <v>105</v>
       </c>
       <c r="C108" t="s">
+        <v>161</v>
+      </c>
+      <c r="D108" t="s">
+        <v>109</v>
+      </c>
+      <c r="E108" t="s">
+        <v>95</v>
+      </c>
+      <c r="F108">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>10</v>
+      </c>
+      <c r="B109" t="s">
+        <v>203</v>
+      </c>
+      <c r="C109" t="s">
+        <v>161</v>
+      </c>
+      <c r="D109" t="s">
+        <v>204</v>
+      </c>
+      <c r="E109" t="s">
+        <v>95</v>
+      </c>
+      <c r="F109">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>10</v>
+      </c>
+      <c r="B110" t="s">
+        <v>205</v>
+      </c>
+      <c r="C110" t="s">
+        <v>161</v>
+      </c>
+      <c r="D110" t="s">
+        <v>206</v>
+      </c>
+      <c r="E110" t="s">
+        <v>95</v>
+      </c>
+      <c r="F110">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>10</v>
+      </c>
+      <c r="B111" t="s">
+        <v>96</v>
+      </c>
+      <c r="C111" t="s">
+        <v>142</v>
+      </c>
+      <c r="D111" t="s">
+        <v>89</v>
+      </c>
+      <c r="E111" t="s">
+        <v>95</v>
+      </c>
+      <c r="F111">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>10</v>
+      </c>
+      <c r="B112" t="s">
+        <v>96</v>
+      </c>
+      <c r="C112" t="s">
+        <v>142</v>
+      </c>
+      <c r="D112" t="s">
+        <v>100</v>
+      </c>
+      <c r="E112" t="s">
+        <v>95</v>
+      </c>
+      <c r="F112">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>20</v>
+      </c>
+      <c r="B113" t="s">
+        <v>96</v>
+      </c>
+      <c r="C113" t="s">
+        <v>161</v>
+      </c>
+      <c r="D113" t="s">
+        <v>89</v>
+      </c>
+      <c r="E113" t="s">
+        <v>95</v>
+      </c>
+      <c r="F113">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>10</v>
+      </c>
+      <c r="B114" t="s">
+        <v>207</v>
+      </c>
+      <c r="C114" t="s">
+        <v>161</v>
+      </c>
+      <c r="D114" t="s">
+        <v>208</v>
+      </c>
+      <c r="E114" t="s">
+        <v>95</v>
+      </c>
+      <c r="F114">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>10</v>
+      </c>
+      <c r="B115" t="s">
+        <v>137</v>
+      </c>
+      <c r="C115" t="s">
+        <v>132</v>
+      </c>
+      <c r="D115" t="s">
+        <v>139</v>
+      </c>
+      <c r="E115" t="s">
+        <v>95</v>
+      </c>
+      <c r="F115">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>10</v>
+      </c>
+      <c r="B116" t="s">
+        <v>137</v>
+      </c>
+      <c r="C116" t="s">
+        <v>132</v>
+      </c>
+      <c r="D116" t="s">
+        <v>292</v>
+      </c>
+      <c r="E116" t="s">
+        <v>95</v>
+      </c>
+      <c r="F116">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>20</v>
+      </c>
+      <c r="B117" t="s">
+        <v>137</v>
+      </c>
+      <c r="C117" t="s">
         <v>90</v>
       </c>
-      <c r="D108" t="s">
+      <c r="D117" t="s">
+        <v>139</v>
+      </c>
+      <c r="E117" t="s">
+        <v>95</v>
+      </c>
+      <c r="F117">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>20</v>
+      </c>
+      <c r="B118" t="s">
+        <v>137</v>
+      </c>
+      <c r="C118" t="s">
         <v>90</v>
       </c>
-      <c r="E108" t="s">
-        <v>95</v>
-      </c>
-      <c r="F108">
+      <c r="D118" t="s">
+        <v>90</v>
+      </c>
+      <c r="E118" t="s">
+        <v>95</v>
+      </c>
+      <c r="F118">
         <v>1</v>
       </c>
     </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>10</v>
+      </c>
+      <c r="B119" t="s">
+        <v>258</v>
+      </c>
+      <c r="C119" t="s">
+        <v>161</v>
+      </c>
+      <c r="D119" t="s">
+        <v>259</v>
+      </c>
+      <c r="E119" t="s">
+        <v>95</v>
+      </c>
+      <c r="F119">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>10</v>
+      </c>
+      <c r="B120" t="s">
+        <v>262</v>
+      </c>
+      <c r="C120" t="s">
+        <v>161</v>
+      </c>
+      <c r="D120" t="s">
+        <v>263</v>
+      </c>
+      <c r="E120" t="s">
+        <v>95</v>
+      </c>
+      <c r="F120">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>10</v>
+      </c>
+      <c r="B121" t="s">
+        <v>264</v>
+      </c>
+      <c r="C121" t="s">
+        <v>161</v>
+      </c>
+      <c r="D121" t="s">
+        <v>265</v>
+      </c>
+      <c r="E121" t="s">
+        <v>95</v>
+      </c>
+      <c r="F121">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>10</v>
+      </c>
+      <c r="B122" t="s">
+        <v>266</v>
+      </c>
+      <c r="C122" t="s">
+        <v>161</v>
+      </c>
+      <c r="D122" t="s">
+        <v>266</v>
+      </c>
+      <c r="E122" t="s">
+        <v>95</v>
+      </c>
+      <c r="F122">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F76" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}"/>
+  <autoFilter ref="A1:F122" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7D90B36-6D7D-4C66-A0D0-AC9375BB2B54}">
+  <dimension ref="A1:E81"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" t="s">
+        <v>255</v>
+      </c>
+      <c r="D1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" t="s">
+        <v>294</v>
+      </c>
+      <c r="D3" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D4" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D5" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C6" t="s">
+        <v>295</v>
+      </c>
+      <c r="D6" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D7" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C8" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>200</v>
+      </c>
+      <c r="B10" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" t="s">
+        <v>332</v>
+      </c>
+      <c r="D10" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>200</v>
+      </c>
+      <c r="B11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" t="s">
+        <v>332</v>
+      </c>
+      <c r="D11" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>200</v>
+      </c>
+      <c r="B12" t="s">
+        <v>267</v>
+      </c>
+      <c r="C12" t="s">
+        <v>332</v>
+      </c>
+      <c r="D12" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C13" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>142</v>
+      </c>
+      <c r="C14" t="s">
+        <v>298</v>
+      </c>
+      <c r="D14" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>161</v>
+      </c>
+      <c r="C15" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>179</v>
+      </c>
+      <c r="B16" t="s">
+        <v>161</v>
+      </c>
+      <c r="C16" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" t="s">
+        <v>161</v>
+      </c>
+      <c r="C17" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>191</v>
+      </c>
+      <c r="B18" t="s">
+        <v>161</v>
+      </c>
+      <c r="C18" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>144</v>
+      </c>
+      <c r="B19" t="s">
+        <v>161</v>
+      </c>
+      <c r="C19" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>205</v>
+      </c>
+      <c r="B20" t="s">
+        <v>161</v>
+      </c>
+      <c r="C20" t="s">
+        <v>304</v>
+      </c>
+      <c r="D20" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" t="s">
+        <v>161</v>
+      </c>
+      <c r="C22" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B23" t="s">
+        <v>161</v>
+      </c>
+      <c r="C23" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>166</v>
+      </c>
+      <c r="B24" t="s">
+        <v>161</v>
+      </c>
+      <c r="C24" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>87</v>
+      </c>
+      <c r="B25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" t="s">
+        <v>311</v>
+      </c>
+      <c r="D25" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" t="s">
+        <v>311</v>
+      </c>
+      <c r="D26" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" t="s">
+        <v>311</v>
+      </c>
+      <c r="D27" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>194</v>
+      </c>
+      <c r="B29" t="s">
+        <v>161</v>
+      </c>
+      <c r="C29" t="s">
+        <v>316</v>
+      </c>
+      <c r="D29" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" t="s">
+        <v>161</v>
+      </c>
+      <c r="C30" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>196</v>
+      </c>
+      <c r="B31" t="s">
+        <v>161</v>
+      </c>
+      <c r="C31" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" t="s">
+        <v>161</v>
+      </c>
+      <c r="C32" t="s">
+        <v>350</v>
+      </c>
+      <c r="D32" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>116</v>
+      </c>
+      <c r="B33" t="s">
+        <v>261</v>
+      </c>
+      <c r="C33" t="s">
+        <v>350</v>
+      </c>
+      <c r="D33" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>147</v>
+      </c>
+      <c r="B34" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>258</v>
+      </c>
+      <c r="B35" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B36" t="s">
+        <v>161</v>
+      </c>
+      <c r="C36" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>207</v>
+      </c>
+      <c r="B37" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>175</v>
+      </c>
+      <c r="B38" t="s">
+        <v>161</v>
+      </c>
+      <c r="C38" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>167</v>
+      </c>
+      <c r="B39" t="s">
+        <v>161</v>
+      </c>
+      <c r="C39" t="s">
+        <v>322</v>
+      </c>
+      <c r="D39" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" t="s">
+        <v>161</v>
+      </c>
+      <c r="C40" t="s">
+        <v>323</v>
+      </c>
+      <c r="D40" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>130</v>
+      </c>
+      <c r="B41" t="s">
+        <v>161</v>
+      </c>
+      <c r="C41" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>173</v>
+      </c>
+      <c r="B42" t="s">
+        <v>161</v>
+      </c>
+      <c r="C42" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>154</v>
+      </c>
+      <c r="B43" t="s">
+        <v>161</v>
+      </c>
+      <c r="C43" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>262</v>
+      </c>
+      <c r="B44" t="s">
+        <v>161</v>
+      </c>
+      <c r="C44" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>264</v>
+      </c>
+      <c r="B45" t="s">
+        <v>161</v>
+      </c>
+      <c r="C45" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B46" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" t="s">
+        <v>313</v>
+      </c>
+      <c r="D46" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>148</v>
+      </c>
+      <c r="B47" t="s">
+        <v>161</v>
+      </c>
+      <c r="C47" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>177</v>
+      </c>
+      <c r="B48" t="s">
+        <v>161</v>
+      </c>
+      <c r="C48" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>257</v>
+      </c>
+      <c r="B49" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" t="s">
+        <v>366</v>
+      </c>
+      <c r="D49" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>134</v>
+      </c>
+      <c r="B50" t="s">
+        <v>161</v>
+      </c>
+      <c r="C50" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>127</v>
+      </c>
+      <c r="B51" t="s">
+        <v>90</v>
+      </c>
+      <c r="C51" t="s">
+        <v>333</v>
+      </c>
+      <c r="D51" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>127</v>
+      </c>
+      <c r="B52" t="s">
+        <v>161</v>
+      </c>
+      <c r="C52" t="s">
+        <v>333</v>
+      </c>
+      <c r="D52" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>118</v>
+      </c>
+      <c r="B53" t="s">
+        <v>161</v>
+      </c>
+      <c r="C53" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>186</v>
+      </c>
+      <c r="B54" t="s">
+        <v>161</v>
+      </c>
+      <c r="C54" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>171</v>
+      </c>
+      <c r="B55" t="s">
+        <v>161</v>
+      </c>
+      <c r="C55" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>162</v>
+      </c>
+      <c r="B56" t="s">
+        <v>292</v>
+      </c>
+      <c r="C56" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>162</v>
+      </c>
+      <c r="B57" t="s">
+        <v>90</v>
+      </c>
+      <c r="C57" t="s">
+        <v>337</v>
+      </c>
+      <c r="D57" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>162</v>
+      </c>
+      <c r="B58" t="s">
+        <v>161</v>
+      </c>
+      <c r="C58" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>169</v>
+      </c>
+      <c r="B59" t="s">
+        <v>161</v>
+      </c>
+      <c r="C59" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>126</v>
+      </c>
+      <c r="B60" t="s">
+        <v>161</v>
+      </c>
+      <c r="C60" t="s">
+        <v>342</v>
+      </c>
+      <c r="D60" t="s">
+        <v>342</v>
+      </c>
+      <c r="E60" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>98</v>
+      </c>
+      <c r="B61" t="s">
+        <v>161</v>
+      </c>
+      <c r="C61" t="s">
+        <v>344</v>
+      </c>
+      <c r="D61" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>106</v>
+      </c>
+      <c r="B62" t="s">
+        <v>161</v>
+      </c>
+      <c r="C62" t="s">
+        <v>354</v>
+      </c>
+      <c r="D62" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>136</v>
+      </c>
+      <c r="B63" t="s">
+        <v>137</v>
+      </c>
+      <c r="C63" t="s">
+        <v>354</v>
+      </c>
+      <c r="D63" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>136</v>
+      </c>
+      <c r="B64" t="s">
+        <v>103</v>
+      </c>
+      <c r="C64" t="s">
+        <v>354</v>
+      </c>
+      <c r="D64" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>136</v>
+      </c>
+      <c r="B65" t="s">
+        <v>197</v>
+      </c>
+      <c r="C65" t="s">
+        <v>354</v>
+      </c>
+      <c r="D65" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>136</v>
+      </c>
+      <c r="B66" t="s">
+        <v>161</v>
+      </c>
+      <c r="C66" t="s">
+        <v>354</v>
+      </c>
+      <c r="D66" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>164</v>
+      </c>
+      <c r="B67" t="s">
+        <v>161</v>
+      </c>
+      <c r="C67" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>203</v>
+      </c>
+      <c r="B68" t="s">
+        <v>161</v>
+      </c>
+      <c r="C68" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>105</v>
+      </c>
+      <c r="B69" t="s">
+        <v>151</v>
+      </c>
+      <c r="C69" t="s">
+        <v>358</v>
+      </c>
+      <c r="D69" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>105</v>
+      </c>
+      <c r="B70" t="s">
+        <v>161</v>
+      </c>
+      <c r="C70" t="s">
+        <v>358</v>
+      </c>
+      <c r="D70" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>181</v>
+      </c>
+      <c r="B71" t="s">
+        <v>182</v>
+      </c>
+      <c r="C71" t="s">
+        <v>352</v>
+      </c>
+      <c r="D71" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>181</v>
+      </c>
+      <c r="B72" t="s">
+        <v>183</v>
+      </c>
+      <c r="C72" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>114</v>
+      </c>
+      <c r="B73" t="s">
+        <v>161</v>
+      </c>
+      <c r="C73" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74" t="s">
+        <v>161</v>
+      </c>
+      <c r="C74" t="s">
+        <v>356</v>
+      </c>
+      <c r="D74" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>152</v>
+      </c>
+      <c r="B75" t="s">
+        <v>161</v>
+      </c>
+      <c r="C75" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>140</v>
+      </c>
+      <c r="B76" t="s">
+        <v>161</v>
+      </c>
+      <c r="C76" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>157</v>
+      </c>
+      <c r="B77" t="s">
+        <v>161</v>
+      </c>
+      <c r="C77" t="s">
+        <v>332</v>
+      </c>
+      <c r="D77" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>150</v>
+      </c>
+      <c r="B78" t="s">
+        <v>161</v>
+      </c>
+      <c r="C78" t="s">
+        <v>354</v>
+      </c>
+      <c r="D78" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>266</v>
+      </c>
+      <c r="B79" t="s">
+        <v>161</v>
+      </c>
+      <c r="C79" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>160</v>
+      </c>
+      <c r="B80" t="s">
+        <v>161</v>
+      </c>
+      <c r="C80" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>192</v>
+      </c>
+      <c r="B81" t="s">
+        <v>161</v>
+      </c>
+      <c r="C81" t="s">
+        <v>346</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D81" xr:uid="{F7D90B36-6D7D-4C66-A0D0-AC9375BB2B54}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Replace unavailable representative card images
</commit_message>
<xml_diff>
--- a/metadata/metadata.xlsx
+++ b/metadata/metadata.xlsx
@@ -15,7 +15,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'archetypes'!$A$1:$F$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'archetype_cards'!$A$1:$D$81</definedName>
   </definedNames>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -5687,7 +5687,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>me02.5-084</t>
+          <t>sv02-045</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>me01-10</t>
+          <t>me01-104</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>me01-10</t>
+          <t>me01-104</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>me01-10</t>
+          <t>me01-104</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>me02.5-111</t>
+          <t>sv10-104</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>me02.5-096</t>
+          <t>sv06-013</t>
         </is>
       </c>
     </row>
@@ -6235,7 +6235,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>me02.5-070</t>
+          <t>sv09-053</t>
         </is>
       </c>
     </row>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>me02.5-076</t>
+          <t>sv09-056</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>me02.5-287</t>
+          <t>sv07-096</t>
         </is>
       </c>
     </row>
@@ -6379,11 +6379,6 @@
           <t>Dusknoir</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>sv06.5-020</t>
-        </is>
-      </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>sv06.5-020</t>
@@ -6403,7 +6398,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>me02.5-267</t>
+          <t>me02-041</t>
         </is>
       </c>
     </row>
@@ -6420,7 +6415,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>me02.5-152</t>
+          <t>sv03-159</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6915,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>me02.5-127</t>
+          <t>me02-058</t>
         </is>
       </c>
     </row>
@@ -6976,7 +6971,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>sv08.5-041</t>
+          <t>sv06.5-022</t>
         </is>
       </c>
     </row>
@@ -7055,6 +7050,11 @@
       <c r="C80" t="inlineStr">
         <is>
           <t>me02-068</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>sv04-123</t>
         </is>
       </c>
     </row>

</xml_diff>